<commit_message>
updated transformations with tuned values and added a few additional ones for wetlands
</commit_message>
<xml_diff>
--- a/data_processing/transformations/UGA mapping NDC with other gov documents 2025_01_10_emp.xlsx
+++ b/data_processing/transformations/UGA mapping NDC with other gov documents 2025_01_10_emp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecmx-my.sharepoint.com/personal/cffuentes_tec_mx/Documents/SISEPUEDE/Uganda/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/ssp_uganda_data/data_processing/transformations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="599" documentId="8_{A2691AC5-F42C-7443-85D9-F492C8AAE86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05EA7457-8512-0F44-856F-CEFE82686F9F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFBE1A4-4D06-F747-9DEC-4A62F007E612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" tabRatio="818" xr2:uid="{1BD21D7C-6458-46D9-BD8C-192871A2CC4A}"/>
+    <workbookView xWindow="780" yWindow="760" windowWidth="33980" windowHeight="20020" tabRatio="818" xr2:uid="{1BD21D7C-6458-46D9-BD8C-192871A2CC4A}"/>
   </bookViews>
   <sheets>
     <sheet name="NDC priority mitigation" sheetId="5" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="349">
   <si>
     <t xml:space="preserve">Sector No. </t>
   </si>
@@ -1337,6 +1337,9 @@
   </si>
   <si>
     <t>This measure is aimed at introducing biogas digesters in schools. Biogas digesters will be fed by waste from bio latrines and used for cooking. The measure has potential to reduce the emissions by 0.0006 MtCO2e by 2030.</t>
+  </si>
+  <si>
+    <t>TX:LNDU:SET_WETLANDS_MINIMUM</t>
   </si>
 </sst>
 </file>
@@ -1786,122 +1789,122 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1942,10 +1945,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2285,11 +2284,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C1" s="112" t="s">
+      <c r="C1" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
       <c r="J1" s="70"/>
     </row>
     <row r="2" spans="1:17" ht="20" x14ac:dyDescent="0.2">
@@ -2337,31 +2336,31 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="81">
+      <c r="A4" s="89">
         <v>1</v>
       </c>
       <c r="B4" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="84" t="s">
+      <c r="C4" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="81" t="s">
+      <c r="D4" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="87" t="s">
+      <c r="E4" s="93" t="s">
         <v>216</v>
       </c>
-      <c r="F4" s="90" t="s">
+      <c r="F4" s="83" t="s">
         <v>310</v>
       </c>
-      <c r="G4" s="106" t="s">
+      <c r="G4" s="105" t="s">
         <v>165</v>
       </c>
-      <c r="H4" s="94">
+      <c r="H4" s="85">
         <v>1.2</v>
       </c>
-      <c r="I4" s="102" t="s">
+      <c r="I4" s="91" t="s">
         <v>163</v>
       </c>
       <c r="J4" s="40" t="s">
@@ -2369,49 +2368,49 @@
       </c>
     </row>
     <row r="5" spans="1:17" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="82"/>
+      <c r="A5" s="99"/>
       <c r="B5" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="85"/>
-      <c r="D5" s="82"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="96"/>
-      <c r="G5" s="107"/>
-      <c r="H5" s="97"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="99"/>
+      <c r="E5" s="103"/>
+      <c r="F5" s="104"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="108"/>
       <c r="I5" s="109"/>
       <c r="J5" s="40" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="82"/>
+      <c r="A6" s="99"/>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="85"/>
-      <c r="D6" s="82"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="96"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="97"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="99"/>
+      <c r="E6" s="103"/>
+      <c r="F6" s="104"/>
+      <c r="G6" s="106"/>
+      <c r="H6" s="108"/>
       <c r="I6" s="109"/>
       <c r="J6" s="40" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="20.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="83"/>
+      <c r="A7" s="90"/>
       <c r="B7" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="86"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="89"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="108"/>
-      <c r="H7" s="95"/>
-      <c r="I7" s="103"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="90"/>
+      <c r="E7" s="94"/>
+      <c r="F7" s="84"/>
+      <c r="G7" s="107"/>
+      <c r="H7" s="86"/>
+      <c r="I7" s="92"/>
       <c r="J7" s="40" t="s">
         <v>306</v>
       </c>
@@ -2458,17 +2457,17 @@
       <c r="C9" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="81" t="s">
+      <c r="D9" s="89" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="104" t="s">
+      <c r="E9" s="81" t="s">
         <v>217</v>
       </c>
-      <c r="F9" s="90" t="s">
+      <c r="F9" s="83" t="s">
         <v>313</v>
       </c>
-      <c r="G9" s="98"/>
-      <c r="H9" s="94">
+      <c r="G9" s="87"/>
+      <c r="H9" s="85">
         <v>0.3</v>
       </c>
       <c r="I9" s="47" t="s">
@@ -2488,11 +2487,11 @@
       <c r="C10" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="83"/>
-      <c r="E10" s="105"/>
-      <c r="F10" s="91"/>
-      <c r="G10" s="99"/>
-      <c r="H10" s="95"/>
+      <c r="D10" s="90"/>
+      <c r="E10" s="82"/>
+      <c r="F10" s="84"/>
+      <c r="G10" s="88"/>
+      <c r="H10" s="86"/>
       <c r="I10" s="47" t="s">
         <v>163</v>
       </c>
@@ -2532,7 +2531,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="60" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A12" s="41">
         <v>1</v>
       </c>
@@ -2661,31 +2660,31 @@
       </c>
     </row>
     <row r="16" spans="1:17" ht="35.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="81">
+      <c r="A16" s="89">
         <v>1</v>
       </c>
       <c r="B16" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="84" t="s">
+      <c r="C16" s="100" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="81" t="s">
+      <c r="D16" s="89" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="87" t="s">
+      <c r="E16" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="90" t="s">
+      <c r="F16" s="83" t="s">
         <v>325</v>
       </c>
-      <c r="G16" s="106" t="s">
+      <c r="G16" s="105" t="s">
         <v>168</v>
       </c>
-      <c r="H16" s="94">
+      <c r="H16" s="85">
         <v>0.3</v>
       </c>
-      <c r="I16" s="102" t="s">
+      <c r="I16" s="91" t="s">
         <v>163</v>
       </c>
       <c r="J16" s="40" t="s">
@@ -2693,17 +2692,17 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="35.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="83"/>
+      <c r="A17" s="90"/>
       <c r="B17" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="86"/>
-      <c r="D17" s="83"/>
-      <c r="E17" s="89"/>
-      <c r="F17" s="91"/>
-      <c r="G17" s="108"/>
-      <c r="H17" s="95"/>
-      <c r="I17" s="103"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="90"/>
+      <c r="E17" s="94"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="107"/>
+      <c r="H17" s="86"/>
+      <c r="I17" s="92"/>
       <c r="J17" s="40" t="s">
         <v>251</v>
       </c>
@@ -2721,19 +2720,19 @@
       <c r="D18" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="87" t="s">
+      <c r="E18" s="93" t="s">
         <v>293</v>
       </c>
-      <c r="F18" s="90" t="s">
+      <c r="F18" s="83" t="s">
         <v>326</v>
       </c>
-      <c r="G18" s="113" t="s">
+      <c r="G18" s="95" t="s">
         <v>321</v>
       </c>
-      <c r="H18" s="94">
+      <c r="H18" s="85">
         <v>0.3</v>
       </c>
-      <c r="I18" s="102" t="s">
+      <c r="I18" s="91" t="s">
         <v>163</v>
       </c>
       <c r="J18" s="40" t="s">
@@ -2753,11 +2752,11 @@
       <c r="D19" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="89"/>
-      <c r="F19" s="91"/>
-      <c r="G19" s="114"/>
-      <c r="H19" s="95"/>
-      <c r="I19" s="103"/>
+      <c r="E19" s="94"/>
+      <c r="F19" s="84"/>
+      <c r="G19" s="96"/>
+      <c r="H19" s="86"/>
+      <c r="I19" s="92"/>
       <c r="J19" s="40" t="s">
         <v>251</v>
       </c>
@@ -2855,7 +2854,7 @@
         <v>163</v>
       </c>
       <c r="J22" s="40" t="s">
-        <v>255</v>
+        <v>348</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="41" customHeight="1" x14ac:dyDescent="0.2">
@@ -2871,19 +2870,19 @@
       <c r="D23" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="E23" s="87" t="s">
+      <c r="E23" s="93" t="s">
         <v>257</v>
       </c>
-      <c r="F23" s="115" t="s">
+      <c r="F23" s="97" t="s">
         <v>329</v>
       </c>
-      <c r="G23" s="113" t="s">
+      <c r="G23" s="95" t="s">
         <v>170</v>
       </c>
-      <c r="H23" s="94">
+      <c r="H23" s="85">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="I23" s="110" t="s">
+      <c r="I23" s="78" t="s">
         <v>163</v>
       </c>
       <c r="J23" s="40" t="s">
@@ -2903,11 +2902,11 @@
       <c r="D24" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="89"/>
-      <c r="F24" s="116"/>
-      <c r="G24" s="114"/>
-      <c r="H24" s="95"/>
-      <c r="I24" s="111"/>
+      <c r="E24" s="94"/>
+      <c r="F24" s="98"/>
+      <c r="G24" s="96"/>
+      <c r="H24" s="86"/>
+      <c r="I24" s="79"/>
       <c r="J24" s="40" t="s">
         <v>331</v>
       </c>
@@ -3137,31 +3136,31 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="81">
+      <c r="A32" s="89">
         <v>3</v>
       </c>
       <c r="B32" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="98" t="s">
+      <c r="C32" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="D32" s="81" t="s">
+      <c r="D32" s="89" t="s">
         <v>41</v>
       </c>
-      <c r="E32" s="104" t="s">
+      <c r="E32" s="81" t="s">
         <v>227</v>
       </c>
-      <c r="F32" s="90" t="s">
+      <c r="F32" s="83" t="s">
         <v>261</v>
       </c>
-      <c r="G32" s="84" t="s">
+      <c r="G32" s="100" t="s">
         <v>190</v>
       </c>
-      <c r="H32" s="94">
+      <c r="H32" s="85">
         <v>1.86</v>
       </c>
-      <c r="I32" s="102" t="s">
+      <c r="I32" s="91" t="s">
         <v>163</v>
       </c>
       <c r="J32" s="40" t="s">
@@ -3169,47 +3168,47 @@
       </c>
     </row>
     <row r="33" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="83"/>
+      <c r="A33" s="90"/>
       <c r="B33" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C33" s="99"/>
-      <c r="D33" s="83"/>
-      <c r="E33" s="105"/>
-      <c r="F33" s="91"/>
-      <c r="G33" s="86"/>
-      <c r="H33" s="95"/>
-      <c r="I33" s="103"/>
+      <c r="C33" s="88"/>
+      <c r="D33" s="90"/>
+      <c r="E33" s="82"/>
+      <c r="F33" s="84"/>
+      <c r="G33" s="102"/>
+      <c r="H33" s="86"/>
+      <c r="I33" s="92"/>
       <c r="J33" s="40" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="81">
+      <c r="A34" s="89">
         <v>3</v>
       </c>
       <c r="B34" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C34" s="98" t="s">
+      <c r="C34" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="D34" s="81" t="s">
+      <c r="D34" s="89" t="s">
         <v>42</v>
       </c>
-      <c r="E34" s="100" t="s">
+      <c r="E34" s="112" t="s">
         <v>228</v>
       </c>
-      <c r="F34" s="92" t="s">
+      <c r="F34" s="114" t="s">
         <v>341</v>
       </c>
-      <c r="G34" s="84" t="s">
+      <c r="G34" s="100" t="s">
         <v>191</v>
       </c>
-      <c r="H34" s="94">
+      <c r="H34" s="85">
         <v>0.54</v>
       </c>
-      <c r="I34" s="102" t="s">
+      <c r="I34" s="91" t="s">
         <v>163</v>
       </c>
       <c r="J34" s="40" t="s">
@@ -3217,17 +3216,17 @@
       </c>
     </row>
     <row r="35" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="83"/>
+      <c r="A35" s="90"/>
       <c r="B35" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C35" s="99"/>
-      <c r="D35" s="83"/>
-      <c r="E35" s="101"/>
-      <c r="F35" s="93"/>
-      <c r="G35" s="86"/>
-      <c r="H35" s="95"/>
-      <c r="I35" s="103"/>
+      <c r="C35" s="88"/>
+      <c r="D35" s="90"/>
+      <c r="E35" s="113"/>
+      <c r="F35" s="115"/>
+      <c r="G35" s="102"/>
+      <c r="H35" s="86"/>
+      <c r="I35" s="92"/>
       <c r="J35" s="40" t="s">
         <v>264</v>
       </c>
@@ -3349,43 +3348,43 @@
       </c>
     </row>
     <row r="40" spans="1:10" ht="23.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="81">
+      <c r="A40" s="89">
         <v>3</v>
       </c>
       <c r="B40" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C40" s="98" t="s">
+      <c r="C40" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="D40" s="81" t="s">
+      <c r="D40" s="89" t="s">
         <v>47</v>
       </c>
-      <c r="E40" s="87" t="s">
+      <c r="E40" s="93" t="s">
         <v>232</v>
       </c>
-      <c r="F40" s="90" t="s">
+      <c r="F40" s="83" t="s">
         <v>346</v>
       </c>
-      <c r="G40" s="84"/>
-      <c r="H40" s="94"/>
-      <c r="I40" s="78"/>
+      <c r="G40" s="100"/>
+      <c r="H40" s="85"/>
+      <c r="I40" s="110"/>
       <c r="J40" s="40" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="23.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="83"/>
+      <c r="A41" s="90"/>
       <c r="B41" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C41" s="99"/>
-      <c r="D41" s="83"/>
-      <c r="E41" s="89"/>
-      <c r="F41" s="91"/>
-      <c r="G41" s="86"/>
-      <c r="H41" s="95"/>
-      <c r="I41" s="80"/>
+      <c r="C41" s="88"/>
+      <c r="D41" s="90"/>
+      <c r="E41" s="94"/>
+      <c r="F41" s="84"/>
+      <c r="G41" s="102"/>
+      <c r="H41" s="86"/>
+      <c r="I41" s="111"/>
       <c r="J41" s="56" t="s">
         <v>269</v>
       </c>
@@ -3555,91 +3554,91 @@
       </c>
     </row>
     <row r="48" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="81">
+      <c r="A48" s="89">
         <v>4</v>
       </c>
       <c r="B48" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="84" t="s">
+      <c r="C48" s="100" t="s">
         <v>240</v>
       </c>
-      <c r="D48" s="81" t="s">
+      <c r="D48" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="E48" s="87" t="s">
+      <c r="E48" s="93" t="s">
         <v>241</v>
       </c>
-      <c r="F48" s="90" t="s">
+      <c r="F48" s="83" t="s">
         <v>277</v>
       </c>
-      <c r="G48" s="84"/>
-      <c r="H48" s="94"/>
-      <c r="I48" s="78"/>
+      <c r="G48" s="100"/>
+      <c r="H48" s="85"/>
+      <c r="I48" s="110"/>
       <c r="J48" s="40" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="82"/>
+      <c r="A49" s="99"/>
       <c r="B49" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C49" s="85"/>
-      <c r="D49" s="82"/>
-      <c r="E49" s="88"/>
-      <c r="F49" s="96"/>
-      <c r="G49" s="85"/>
-      <c r="H49" s="97"/>
-      <c r="I49" s="79"/>
+      <c r="C49" s="101"/>
+      <c r="D49" s="99"/>
+      <c r="E49" s="103"/>
+      <c r="F49" s="104"/>
+      <c r="G49" s="101"/>
+      <c r="H49" s="108"/>
+      <c r="I49" s="116"/>
       <c r="J49" s="40" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="82"/>
+      <c r="A50" s="99"/>
       <c r="B50" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C50" s="85"/>
-      <c r="D50" s="82"/>
-      <c r="E50" s="88"/>
-      <c r="F50" s="96"/>
-      <c r="G50" s="85"/>
-      <c r="H50" s="97"/>
-      <c r="I50" s="79"/>
+      <c r="C50" s="101"/>
+      <c r="D50" s="99"/>
+      <c r="E50" s="103"/>
+      <c r="F50" s="104"/>
+      <c r="G50" s="101"/>
+      <c r="H50" s="108"/>
+      <c r="I50" s="116"/>
       <c r="J50" s="40" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="82"/>
+      <c r="A51" s="99"/>
       <c r="B51" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C51" s="85"/>
-      <c r="D51" s="82"/>
-      <c r="E51" s="88"/>
-      <c r="F51" s="96"/>
-      <c r="G51" s="85"/>
-      <c r="H51" s="97"/>
-      <c r="I51" s="79"/>
+      <c r="C51" s="101"/>
+      <c r="D51" s="99"/>
+      <c r="E51" s="103"/>
+      <c r="F51" s="104"/>
+      <c r="G51" s="101"/>
+      <c r="H51" s="108"/>
+      <c r="I51" s="116"/>
       <c r="J51" s="40" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="83"/>
+      <c r="A52" s="90"/>
       <c r="B52" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C52" s="86"/>
-      <c r="D52" s="83"/>
-      <c r="E52" s="89"/>
-      <c r="F52" s="91"/>
-      <c r="G52" s="86"/>
-      <c r="H52" s="95"/>
-      <c r="I52" s="80"/>
+      <c r="C52" s="102"/>
+      <c r="D52" s="90"/>
+      <c r="E52" s="94"/>
+      <c r="F52" s="84"/>
+      <c r="G52" s="102"/>
+      <c r="H52" s="86"/>
+      <c r="I52" s="111"/>
       <c r="J52" s="40" t="s">
         <v>276</v>
       </c>
@@ -3759,6 +3758,54 @@
   </sheetData>
   <autoFilter ref="A3:I56" xr:uid="{BFF41CA7-F102-4D3E-A927-D5D9825C06C8}"/>
   <mergeCells count="64">
+    <mergeCell ref="I48:I52"/>
+    <mergeCell ref="A48:A52"/>
+    <mergeCell ref="C48:C52"/>
+    <mergeCell ref="D48:D52"/>
+    <mergeCell ref="E48:E52"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="H34:H35"/>
+    <mergeCell ref="F48:F52"/>
+    <mergeCell ref="G48:G52"/>
+    <mergeCell ref="H48:H52"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="G34:G35"/>
+    <mergeCell ref="I32:I33"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="H40:H41"/>
+    <mergeCell ref="I40:I41"/>
+    <mergeCell ref="H32:H33"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="F4:F7"/>
+    <mergeCell ref="G4:G7"/>
+    <mergeCell ref="H4:H7"/>
+    <mergeCell ref="I4:I7"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
     <mergeCell ref="I23:I24"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="E9:E10"/>
@@ -3775,54 +3822,6 @@
     <mergeCell ref="E23:E24"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="G23:G24"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="D4:D7"/>
-    <mergeCell ref="E4:E7"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="F4:F7"/>
-    <mergeCell ref="G4:G7"/>
-    <mergeCell ref="H4:H7"/>
-    <mergeCell ref="I4:I7"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="G32:G33"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="G34:G35"/>
-    <mergeCell ref="I32:I33"/>
-    <mergeCell ref="G40:G41"/>
-    <mergeCell ref="H40:H41"/>
-    <mergeCell ref="I40:I41"/>
-    <mergeCell ref="H32:H33"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="F34:F35"/>
-    <mergeCell ref="H34:H35"/>
-    <mergeCell ref="F48:F52"/>
-    <mergeCell ref="G48:G52"/>
-    <mergeCell ref="H48:H52"/>
-    <mergeCell ref="I48:I52"/>
-    <mergeCell ref="A48:A52"/>
-    <mergeCell ref="C48:C52"/>
-    <mergeCell ref="D48:D52"/>
-    <mergeCell ref="E48:E52"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated transformations and added new bounds for variables
</commit_message>
<xml_diff>
--- a/data_processing/transformations/UGA mapping NDC with other gov documents 2025_01_10_emp.xlsx
+++ b/data_processing/transformations/UGA mapping NDC with other gov documents 2025_01_10_emp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/ssp_uganda_data/data_processing/transformations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFBE1A4-4D06-F747-9DEC-4A62F007E612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A8D0FD-A122-C24D-9273-7568DB762008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="760" windowWidth="33980" windowHeight="20020" tabRatio="818" xr2:uid="{1BD21D7C-6458-46D9-BD8C-192871A2CC4A}"/>
+    <workbookView xWindow="-1200" yWindow="760" windowWidth="33980" windowHeight="20020" tabRatio="818" xr2:uid="{1BD21D7C-6458-46D9-BD8C-192871A2CC4A}"/>
   </bookViews>
   <sheets>
     <sheet name="NDC priority mitigation" sheetId="5" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="353">
   <si>
     <t xml:space="preserve">Sector No. </t>
   </si>
@@ -1341,6 +1341,18 @@
   <si>
     <t>TX:LNDU:SET_WETLANDS_MINIMUM</t>
   </si>
+  <si>
+    <t>Inc reforestation</t>
+  </si>
+  <si>
+    <t>Increase sequestration</t>
+  </si>
+  <si>
+    <t>reduce demand for biomass--passed in SCOE</t>
+  </si>
+  <si>
+    <t>TX:SCOE:INC_EFFICIENCY_ENERGY</t>
+  </si>
 </sst>
 </file>
 
@@ -1349,9 +1361,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1576,55 +1595,55 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1632,38 +1651,38 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1672,70 +1691,70 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1744,22 +1763,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1771,43 +1790,43 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1828,106 +1847,109 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="17" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2530,6 +2552,9 @@
       <c r="J11" s="40" t="s">
         <v>255</v>
       </c>
+      <c r="K11" s="23" t="s">
+        <v>350</v>
+      </c>
     </row>
     <row r="12" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A12" s="41">
@@ -2562,6 +2587,9 @@
       <c r="J12" s="40" t="s">
         <v>255</v>
       </c>
+      <c r="K12" s="23" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="13" spans="1:17" ht="180" x14ac:dyDescent="0.2">
       <c r="A13" s="41">
@@ -2593,6 +2621,9 @@
       </c>
       <c r="J13" s="40" t="s">
         <v>255</v>
+      </c>
+      <c r="K13" s="23" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="75" x14ac:dyDescent="0.2">
@@ -3131,8 +3162,8 @@
       <c r="I31" s="47" t="s">
         <v>163</v>
       </c>
-      <c r="J31" s="77" t="s">
-        <v>339</v>
+      <c r="J31" s="125" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3823,7 +3854,7 @@
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="G23:G24"/>
   </mergeCells>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>

</xml_diff>